<commit_message>
Update Deliverable 9 in completed workbook with 465s technical demonstration video
</commit_message>
<xml_diff>
--- a/submission/IncuBrix_PS03_Submission_Evaluation_Batch_Moderation_Workbook_COMPLETED.xlsx
+++ b/submission/IncuBrix_PS03_Submission_Evaluation_Batch_Moderation_Workbook_COMPLETED.xlsx
@@ -1588,12 +1588,12 @@
       </c>
       <c r="D13" s="19" t="inlineStr">
         <is>
-          <t>submission/artifacts/final_draft.mp4</t>
+          <t>submission/TECHNICAL_DEMONSTRATION_PS03.mp4, submission/TECHNICAL_DEMONSTRATION_METADATA.md</t>
         </is>
       </c>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>20-second 1280x720 30fps H.264/AAC draft video demonstrating multi-scene composition, typography, and captions</t>
+          <t>465.0s (7m 45s) continuous technical walkthrough at 1280x720 30fps H.264/AAC with synchronized audio covering all 10 rubric sections; plus demonstrated final_draft.mp4</t>
         </is>
       </c>
       <c r="F13" s="48" t="str"/>

</xml_diff>